<commit_message>
reset arn label to weekly
</commit_message>
<xml_diff>
--- a/ARN_Template.xlsx
+++ b/ARN_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://actmaxmy-my.sharepoint.com/personal/fakrul_hussin_actmax_com/Documents/Barcode/Barcode_Printing_Node/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="55" documentId="13_ncr:1_{3DBAF157-7925-4AAA-8D37-4A9067F6F593}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D8F2CFF0-7CE8-41B0-B787-8675354541F2}"/>
+  <xr:revisionPtr revIDLastSave="60" documentId="13_ncr:1_{3DBAF157-7925-4AAA-8D37-4A9067F6F593}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17ECD49A-8E03-4F25-9776-E869AE7CC39F}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{91116337-D2E0-49FF-BAB3-CCBCE167A5E6}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>ARN PartNo</t>
   </si>
@@ -51,6 +51,15 @@
   </si>
   <si>
     <t>Purchase Order</t>
+  </si>
+  <si>
+    <t>K2003</t>
+  </si>
+  <si>
+    <t>P0123</t>
+  </si>
+  <si>
+    <t>test123</t>
   </si>
 </sst>
 </file>
@@ -488,10 +497,18 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="1">
+        <v>123</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>

</xml_diff>

<commit_message>
add workflow separation and printer setup page
</commit_message>
<xml_diff>
--- a/ARN_Template.xlsx
+++ b/ARN_Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://actmaxmy-my.sharepoint.com/personal/fakrul_hussin_actmax_com/Documents/Barcode/Barcode_Printing_Node/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="60" documentId="13_ncr:1_{3DBAF157-7925-4AAA-8D37-4A9067F6F593}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17ECD49A-8E03-4F25-9776-E869AE7CC39F}"/>
+  <xr:revisionPtr revIDLastSave="65" documentId="13_ncr:1_{3DBAF157-7925-4AAA-8D37-4A9067F6F593}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{521414CA-36CF-4819-AF90-32AC2AE9B8A1}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{91116337-D2E0-49FF-BAB3-CCBCE167A5E6}"/>
   </bookViews>
@@ -53,13 +53,13 @@
     <t>Purchase Order</t>
   </si>
   <si>
-    <t>K2003</t>
+    <t>test001</t>
   </si>
   <si>
-    <t>P0123</t>
+    <t>qwerty</t>
   </si>
   <si>
-    <t>test123</t>
+    <t>N/A</t>
   </si>
 </sst>
 </file>
@@ -137,10 +137,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -498,16 +494,16 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B2" s="1">
-        <v>123</v>
+        <v>3</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">

</xml_diff>